<commit_message>
Cập nhật biên bản nghiệm thu GD1: BUG_UI_107 đã đóng, 5/5 DS đạt
- Thêm extract_nghiemthu_gd1.py để trích lại dữ liệu từ file QA, thay cho
  việc sửa tay data_nghiemthu_gd1.json.
- BUG_UI_107 (DS_22) chuyển Fixed, Retest Pass ngày 17/09/2026 kèm bằng chứng
  => DS_22 đủ 4 điều kiện, toàn bộ 5 màn hình và 12 tính năng đạt nghiệm thu.
- Mục tiêu chí, kết luận và vấn đề tồn đọng sinh theo dữ liệu thay vì text cố
  định, nên tự đổi khi trạng thái lỗi thay đổi.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JSytd29s9p6EiQAewGnqRv
</commit_message>
<xml_diff>
--- a/BaoCao_NghiemThu_GD1.xlsx
+++ b/BaoCao_NghiemThu_GD1.xlsx
@@ -19,7 +19,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,19 +76,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C62828"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="001F3A5F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00C62828"/>
       <sz val="11"/>
     </font>
     <font>
@@ -106,12 +94,6 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00C62828"/>
-      <sz val="10.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="10.5"/>
     </font>
@@ -122,7 +104,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -162,11 +144,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9F0DD"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FBE3E3"/>
       </patternFill>
     </fill>
   </fills>
@@ -240,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -289,35 +266,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -327,29 +294,26 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1423,22 +1387,22 @@
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>1 lỗi đang mở</t>
+          <t>0 lỗi đang mở</t>
         </is>
       </c>
       <c r="F24" s="16" t="n"/>
-      <c r="G24" s="22" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="H24" s="23" t="n"/>
-      <c r="I24" s="23" t="n"/>
-      <c r="J24" s="23" t="n"/>
-      <c r="K24" s="23" t="n"/>
-      <c r="L24" s="23" t="n"/>
-      <c r="M24" s="23" t="n"/>
-      <c r="N24" s="23" t="n"/>
+      <c r="G24" s="20" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="H24" s="21" t="n"/>
+      <c r="I24" s="21" t="n"/>
+      <c r="J24" s="21" t="n"/>
+      <c r="K24" s="21" t="n"/>
+      <c r="L24" s="21" t="n"/>
+      <c r="M24" s="21" t="n"/>
+      <c r="N24" s="21" t="n"/>
     </row>
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="13" t="inlineStr">
@@ -1459,22 +1423,22 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>1 lỗi Critical/High đang mở</t>
+          <t>0 lỗi Critical/High đang mở</t>
         </is>
       </c>
       <c r="F25" s="11" t="n"/>
-      <c r="G25" s="22" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="H25" s="23" t="n"/>
-      <c r="I25" s="23" t="n"/>
-      <c r="J25" s="23" t="n"/>
-      <c r="K25" s="23" t="n"/>
-      <c r="L25" s="23" t="n"/>
-      <c r="M25" s="23" t="n"/>
-      <c r="N25" s="23" t="n"/>
+      <c r="G25" s="20" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="H25" s="21" t="n"/>
+      <c r="I25" s="21" t="n"/>
+      <c r="J25" s="21" t="n"/>
+      <c r="K25" s="21" t="n"/>
+      <c r="L25" s="21" t="n"/>
+      <c r="M25" s="21" t="n"/>
+      <c r="N25" s="21" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
       <c r="A26" s="14" t="inlineStr">
@@ -1495,22 +1459,22 @@
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>18/19 lỗi đạt Retest Pass</t>
+          <t>19/19 lỗi đạt Retest Pass</t>
         </is>
       </c>
       <c r="F26" s="16" t="n"/>
-      <c r="G26" s="22" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="H26" s="23" t="n"/>
-      <c r="I26" s="23" t="n"/>
-      <c r="J26" s="23" t="n"/>
-      <c r="K26" s="23" t="n"/>
-      <c r="L26" s="23" t="n"/>
-      <c r="M26" s="23" t="n"/>
-      <c r="N26" s="23" t="n"/>
+      <c r="G26" s="20" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="21" t="n"/>
+      <c r="J26" s="21" t="n"/>
+      <c r="K26" s="21" t="n"/>
+      <c r="L26" s="21" t="n"/>
+      <c r="M26" s="21" t="n"/>
+      <c r="N26" s="21" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
       <c r="A27" s="13" t="inlineStr">
@@ -1660,7 +1624,7 @@
         </is>
       </c>
       <c r="B32" s="11" t="n"/>
-      <c r="C32" s="24" t="n">
+      <c r="C32" s="22" t="n">
         <v>5</v>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -1669,7 +1633,7 @@
         </is>
       </c>
       <c r="E32" s="11" t="n"/>
-      <c r="F32" s="24" t="n">
+      <c r="F32" s="22" t="n">
         <v>12</v>
       </c>
       <c r="G32" s="10" t="inlineStr">
@@ -1678,7 +1642,7 @@
         </is>
       </c>
       <c r="H32" s="11" t="n"/>
-      <c r="I32" s="24" t="n">
+      <c r="I32" s="22" t="n">
         <v>19</v>
       </c>
       <c r="J32" s="10" t="inlineStr">
@@ -1687,8 +1651,8 @@
         </is>
       </c>
       <c r="K32" s="11" t="n"/>
-      <c r="L32" s="24" t="n">
-        <v>18</v>
+      <c r="L32" s="22" t="n">
+        <v>19</v>
       </c>
       <c r="M32" s="13" t="n"/>
       <c r="N32" s="13" t="n"/>
@@ -1700,8 +1664,8 @@
         </is>
       </c>
       <c r="B33" s="16" t="n"/>
-      <c r="C33" s="25" t="n">
-        <v>4</v>
+      <c r="C33" s="23" t="n">
+        <v>5</v>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
@@ -1709,8 +1673,8 @@
         </is>
       </c>
       <c r="E33" s="16" t="n"/>
-      <c r="F33" s="26" t="n">
-        <v>1</v>
+      <c r="F33" s="23" t="n">
+        <v>0</v>
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
@@ -1718,8 +1682,8 @@
         </is>
       </c>
       <c r="H33" s="16" t="n"/>
-      <c r="I33" s="26" t="n">
-        <v>1</v>
+      <c r="I33" s="23" t="n">
+        <v>0</v>
       </c>
       <c r="J33" s="15" t="inlineStr">
         <is>
@@ -1727,8 +1691,8 @@
         </is>
       </c>
       <c r="K33" s="16" t="n"/>
-      <c r="L33" s="26" t="n">
-        <v>1</v>
+      <c r="L33" s="23" t="n">
+        <v>0</v>
       </c>
       <c r="M33" s="14" t="n"/>
       <c r="N33" s="14" t="n"/>
@@ -1740,8 +1704,8 @@
         </is>
       </c>
       <c r="B34" s="11" t="n"/>
-      <c r="C34" s="24" t="n">
-        <v>18</v>
+      <c r="C34" s="22" t="n">
+        <v>19</v>
       </c>
       <c r="D34" s="10" t="inlineStr">
         <is>
@@ -1749,8 +1713,8 @@
         </is>
       </c>
       <c r="E34" s="11" t="n"/>
-      <c r="F34" s="24" t="n">
-        <v>1</v>
+      <c r="F34" s="22" t="n">
+        <v>0</v>
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
@@ -1758,7 +1722,7 @@
         </is>
       </c>
       <c r="H34" s="11" t="n"/>
-      <c r="I34" s="24" t="n">
+      <c r="I34" s="22" t="n">
         <v>29</v>
       </c>
       <c r="J34" s="10" t="inlineStr">
@@ -1767,9 +1731,9 @@
         </is>
       </c>
       <c r="K34" s="11" t="n"/>
-      <c r="L34" s="24" t="inlineStr">
-        <is>
-          <t>4/5</t>
+      <c r="L34" s="22" t="inlineStr">
+        <is>
+          <t>5/5</t>
         </is>
       </c>
       <c r="M34" s="13" t="n"/>
@@ -1884,7 +1848,7 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="D38" s="27" t="n">
+      <c r="D38" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E38" s="13" t="n">
@@ -1903,10 +1867,10 @@
       <c r="H38" s="13" t="n">
         <v>6</v>
       </c>
-      <c r="I38" s="28" t="n">
+      <c r="I38" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="J38" s="28" t="n">
+      <c r="J38" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K38" s="13" t="inlineStr">
@@ -1919,12 +1883,12 @@
           <t>15/09/2026</t>
         </is>
       </c>
-      <c r="M38" s="29" t="inlineStr">
+      <c r="M38" s="26" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="N38" s="30" t="n"/>
+      <c r="N38" s="27" t="n"/>
     </row>
     <row r="39" ht="34" customHeight="1">
       <c r="A39" s="14" t="inlineStr">
@@ -1942,7 +1906,7 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="D39" s="31" t="n">
+      <c r="D39" s="28" t="n">
         <v>1</v>
       </c>
       <c r="E39" s="14" t="n">
@@ -1961,10 +1925,10 @@
       <c r="H39" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="I39" s="28" t="n">
+      <c r="I39" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="J39" s="28" t="n">
+      <c r="J39" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K39" s="14" t="inlineStr">
@@ -1977,12 +1941,12 @@
           <t>03/07/2026</t>
         </is>
       </c>
-      <c r="M39" s="29" t="inlineStr">
+      <c r="M39" s="26" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="N39" s="30" t="n"/>
+      <c r="N39" s="27" t="n"/>
     </row>
     <row r="40" ht="34" customHeight="1">
       <c r="A40" s="13" t="inlineStr">
@@ -2000,7 +1964,7 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="D40" s="27" t="n">
+      <c r="D40" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="13" t="n">
@@ -2019,10 +1983,10 @@
       <c r="H40" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="I40" s="28" t="n">
+      <c r="I40" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="J40" s="28" t="n">
+      <c r="J40" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K40" s="13" t="inlineStr">
@@ -2035,12 +1999,12 @@
           <t>09/07/2026</t>
         </is>
       </c>
-      <c r="M40" s="29" t="inlineStr">
+      <c r="M40" s="26" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="N40" s="30" t="n"/>
+      <c r="N40" s="27" t="n"/>
     </row>
     <row r="41" ht="34" customHeight="1">
       <c r="A41" s="14" t="inlineStr">
@@ -2058,7 +2022,7 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="D41" s="31" t="n">
+      <c r="D41" s="28" t="n">
         <v>1</v>
       </c>
       <c r="E41" s="14" t="n">
@@ -2071,21 +2035,21 @@
       </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
-          <t>Còn 1 lỗi đang mở; Còn 1 lỗi Critical/High chưa đóng</t>
+          <t>Đủ 4 điều kiện nghiệm thu</t>
         </is>
       </c>
       <c r="H41" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="I41" s="22" t="n">
-        <v>1</v>
-      </c>
-      <c r="J41" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="I41" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="25" t="n">
+        <v>0</v>
       </c>
       <c r="K41" s="14" t="inlineStr">
         <is>
-          <t>1/2</t>
+          <t>2/2</t>
         </is>
       </c>
       <c r="L41" s="14" t="inlineStr">
@@ -2093,12 +2057,12 @@
           <t>10/09/2026</t>
         </is>
       </c>
-      <c r="M41" s="32" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="N41" s="30" t="n"/>
+      <c r="M41" s="26" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="N41" s="27" t="n"/>
     </row>
     <row r="42" ht="34" customHeight="1">
       <c r="A42" s="13" t="inlineStr">
@@ -2116,7 +2080,7 @@
           <t>Hoàn thành</t>
         </is>
       </c>
-      <c r="D42" s="27" t="n">
+      <c r="D42" s="24" t="n">
         <v>1</v>
       </c>
       <c r="E42" s="13" t="n">
@@ -2135,10 +2099,10 @@
       <c r="H42" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="I42" s="28" t="n">
+      <c r="I42" s="25" t="n">
         <v>0</v>
       </c>
-      <c r="J42" s="28" t="n">
+      <c r="J42" s="25" t="n">
         <v>0</v>
       </c>
       <c r="K42" s="13" t="inlineStr">
@@ -2151,12 +2115,12 @@
           <t>16/09/2026</t>
         </is>
       </c>
-      <c r="M42" s="29" t="inlineStr">
+      <c r="M42" s="26" t="inlineStr">
         <is>
           <t>ĐẠT</t>
         </is>
       </c>
-      <c r="N42" s="30" t="n"/>
+      <c r="N42" s="27" t="n"/>
     </row>
     <row r="43" ht="8" customHeight="1"/>
     <row r="44" ht="24" customHeight="1">
@@ -2360,7 +2324,7 @@
         </is>
       </c>
       <c r="L48" s="21" t="n"/>
-      <c r="M48" s="33" t="inlineStr"/>
+      <c r="M48" s="29" t="inlineStr"/>
       <c r="N48" s="16" t="n"/>
     </row>
     <row r="49" ht="24" customHeight="1">
@@ -2464,7 +2428,7 @@
         </is>
       </c>
       <c r="L50" s="21" t="n"/>
-      <c r="M50" s="33" t="inlineStr"/>
+      <c r="M50" s="29" t="inlineStr"/>
       <c r="N50" s="16" t="n"/>
     </row>
     <row r="51" ht="24" customHeight="1">
@@ -2568,7 +2532,7 @@
         </is>
       </c>
       <c r="L52" s="21" t="n"/>
-      <c r="M52" s="33" t="inlineStr"/>
+      <c r="M52" s="29" t="inlineStr"/>
       <c r="N52" s="16" t="n"/>
     </row>
     <row r="53" ht="24" customHeight="1">
@@ -2666,17 +2630,13 @@
           <t>24/07/2026</t>
         </is>
       </c>
-      <c r="K54" s="22" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="L54" s="23" t="n"/>
-      <c r="M54" s="33" t="inlineStr">
-        <is>
-          <t>Chặn bởi lỗi còn mở trên màn hình</t>
-        </is>
-      </c>
+      <c r="K54" s="20" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="L54" s="21" t="n"/>
+      <c r="M54" s="29" t="inlineStr"/>
       <c r="N54" s="16" t="n"/>
     </row>
     <row r="55" ht="24" customHeight="1">
@@ -2722,17 +2682,13 @@
           <t>16/09/2026</t>
         </is>
       </c>
-      <c r="K55" s="22" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="L55" s="23" t="n"/>
-      <c r="M55" s="19" t="inlineStr">
-        <is>
-          <t>Chặn bởi lỗi còn mở trên màn hình</t>
-        </is>
-      </c>
+      <c r="K55" s="20" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="L55" s="21" t="n"/>
+      <c r="M55" s="19" t="inlineStr"/>
       <c r="N55" s="11" t="n"/>
     </row>
     <row r="56" ht="24" customHeight="1">
@@ -2778,17 +2734,13 @@
           <t>14/08/2026</t>
         </is>
       </c>
-      <c r="K56" s="22" t="inlineStr">
-        <is>
-          <t>CHƯA ĐẠT</t>
-        </is>
-      </c>
-      <c r="L56" s="23" t="n"/>
-      <c r="M56" s="33" t="inlineStr">
-        <is>
-          <t>Chặn bởi lỗi còn mở trên màn hình</t>
-        </is>
-      </c>
+      <c r="K56" s="20" t="inlineStr">
+        <is>
+          <t>ĐẠT</t>
+        </is>
+      </c>
+      <c r="L56" s="21" t="n"/>
+      <c r="M56" s="29" t="inlineStr"/>
       <c r="N56" s="16" t="n"/>
     </row>
     <row r="57" ht="24" customHeight="1">
@@ -2892,7 +2844,7 @@
         </is>
       </c>
       <c r="L58" s="21" t="n"/>
-      <c r="M58" s="33" t="inlineStr"/>
+      <c r="M58" s="29" t="inlineStr"/>
       <c r="N58" s="16" t="n"/>
     </row>
     <row r="59" ht="8" customHeight="1"/>
@@ -3009,24 +2961,24 @@
       </c>
     </row>
     <row r="63" ht="22" customHeight="1">
-      <c r="A63" s="34" t="inlineStr">
+      <c r="A63" s="30" t="inlineStr">
         <is>
           <t>DS_04 — Trang Tìm kiếm   (6 lỗi: 6 đã xử lý, 0 đang mở)</t>
         </is>
       </c>
-      <c r="B63" s="35" t="n"/>
-      <c r="C63" s="35" t="n"/>
-      <c r="D63" s="35" t="n"/>
-      <c r="E63" s="35" t="n"/>
-      <c r="F63" s="35" t="n"/>
-      <c r="G63" s="35" t="n"/>
-      <c r="H63" s="35" t="n"/>
-      <c r="I63" s="35" t="n"/>
-      <c r="J63" s="35" t="n"/>
-      <c r="K63" s="35" t="n"/>
-      <c r="L63" s="35" t="n"/>
-      <c r="M63" s="35" t="n"/>
-      <c r="N63" s="35" t="n"/>
+      <c r="B63" s="31" t="n"/>
+      <c r="C63" s="31" t="n"/>
+      <c r="D63" s="31" t="n"/>
+      <c r="E63" s="31" t="n"/>
+      <c r="F63" s="31" t="n"/>
+      <c r="G63" s="31" t="n"/>
+      <c r="H63" s="31" t="n"/>
+      <c r="I63" s="31" t="n"/>
+      <c r="J63" s="31" t="n"/>
+      <c r="K63" s="31" t="n"/>
+      <c r="L63" s="31" t="n"/>
+      <c r="M63" s="31" t="n"/>
+      <c r="N63" s="31" t="n"/>
     </row>
     <row r="64" ht="30" customHeight="1">
       <c r="A64" s="13" t="inlineStr">
@@ -3464,24 +3416,24 @@
       </c>
     </row>
     <row r="70" ht="22" customHeight="1">
-      <c r="A70" s="34" t="inlineStr">
+      <c r="A70" s="30" t="inlineStr">
         <is>
           <t>DS_05 — Trang Cẩm nang nghề   (3 lỗi: 3 đã xử lý, 0 đang mở)</t>
         </is>
       </c>
-      <c r="B70" s="35" t="n"/>
-      <c r="C70" s="35" t="n"/>
-      <c r="D70" s="35" t="n"/>
-      <c r="E70" s="35" t="n"/>
-      <c r="F70" s="35" t="n"/>
-      <c r="G70" s="35" t="n"/>
-      <c r="H70" s="35" t="n"/>
-      <c r="I70" s="35" t="n"/>
-      <c r="J70" s="35" t="n"/>
-      <c r="K70" s="35" t="n"/>
-      <c r="L70" s="35" t="n"/>
-      <c r="M70" s="35" t="n"/>
-      <c r="N70" s="35" t="n"/>
+      <c r="B70" s="31" t="n"/>
+      <c r="C70" s="31" t="n"/>
+      <c r="D70" s="31" t="n"/>
+      <c r="E70" s="31" t="n"/>
+      <c r="F70" s="31" t="n"/>
+      <c r="G70" s="31" t="n"/>
+      <c r="H70" s="31" t="n"/>
+      <c r="I70" s="31" t="n"/>
+      <c r="J70" s="31" t="n"/>
+      <c r="K70" s="31" t="n"/>
+      <c r="L70" s="31" t="n"/>
+      <c r="M70" s="31" t="n"/>
+      <c r="N70" s="31" t="n"/>
     </row>
     <row r="71" ht="30" customHeight="1">
       <c r="A71" s="13" t="inlineStr">
@@ -3700,24 +3652,24 @@
       </c>
     </row>
     <row r="74" ht="22" customHeight="1">
-      <c r="A74" s="34" t="inlineStr">
+      <c r="A74" s="30" t="inlineStr">
         <is>
           <t>DS_21 — Trang Đăng nhập   (3 lỗi: 3 đã xử lý, 0 đang mở)</t>
         </is>
       </c>
-      <c r="B74" s="35" t="n"/>
-      <c r="C74" s="35" t="n"/>
-      <c r="D74" s="35" t="n"/>
-      <c r="E74" s="35" t="n"/>
-      <c r="F74" s="35" t="n"/>
-      <c r="G74" s="35" t="n"/>
-      <c r="H74" s="35" t="n"/>
-      <c r="I74" s="35" t="n"/>
-      <c r="J74" s="35" t="n"/>
-      <c r="K74" s="35" t="n"/>
-      <c r="L74" s="35" t="n"/>
-      <c r="M74" s="35" t="n"/>
-      <c r="N74" s="35" t="n"/>
+      <c r="B74" s="31" t="n"/>
+      <c r="C74" s="31" t="n"/>
+      <c r="D74" s="31" t="n"/>
+      <c r="E74" s="31" t="n"/>
+      <c r="F74" s="31" t="n"/>
+      <c r="G74" s="31" t="n"/>
+      <c r="H74" s="31" t="n"/>
+      <c r="I74" s="31" t="n"/>
+      <c r="J74" s="31" t="n"/>
+      <c r="K74" s="31" t="n"/>
+      <c r="L74" s="31" t="n"/>
+      <c r="M74" s="31" t="n"/>
+      <c r="N74" s="31" t="n"/>
     </row>
     <row r="75" ht="30" customHeight="1">
       <c r="A75" s="14" t="inlineStr">
@@ -3936,24 +3888,24 @@
       </c>
     </row>
     <row r="78" ht="22" customHeight="1">
-      <c r="A78" s="34" t="inlineStr">
-        <is>
-          <t>DS_22 — Trang Đăng ký   (2 lỗi: 1 đã xử lý, 1 đang mở)</t>
-        </is>
-      </c>
-      <c r="B78" s="35" t="n"/>
-      <c r="C78" s="35" t="n"/>
-      <c r="D78" s="35" t="n"/>
-      <c r="E78" s="35" t="n"/>
-      <c r="F78" s="35" t="n"/>
-      <c r="G78" s="35" t="n"/>
-      <c r="H78" s="35" t="n"/>
-      <c r="I78" s="35" t="n"/>
-      <c r="J78" s="35" t="n"/>
-      <c r="K78" s="35" t="n"/>
-      <c r="L78" s="35" t="n"/>
-      <c r="M78" s="35" t="n"/>
-      <c r="N78" s="35" t="n"/>
+      <c r="A78" s="30" t="inlineStr">
+        <is>
+          <t>DS_22 — Trang Đăng ký   (2 lỗi: 2 đã xử lý, 0 đang mở)</t>
+        </is>
+      </c>
+      <c r="B78" s="31" t="n"/>
+      <c r="C78" s="31" t="n"/>
+      <c r="D78" s="31" t="n"/>
+      <c r="E78" s="31" t="n"/>
+      <c r="F78" s="31" t="n"/>
+      <c r="G78" s="31" t="n"/>
+      <c r="H78" s="31" t="n"/>
+      <c r="I78" s="31" t="n"/>
+      <c r="J78" s="31" t="n"/>
+      <c r="K78" s="31" t="n"/>
+      <c r="L78" s="31" t="n"/>
+      <c r="M78" s="31" t="n"/>
+      <c r="N78" s="31" t="n"/>
     </row>
     <row r="79" ht="30" customHeight="1">
       <c r="A79" s="13" t="inlineStr">
@@ -4048,7 +4000,7 @@
           <t>YC_06</t>
         </is>
       </c>
-      <c r="E80" s="36" t="inlineStr">
+      <c r="E80" s="14" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
@@ -4080,17 +4032,17 @@
       </c>
       <c r="K80" s="14" t="inlineStr">
         <is>
-          <t>Chưa retest</t>
+          <t>Pass</t>
         </is>
       </c>
       <c r="L80" s="14" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="M80" s="22" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>17/09/2026</t>
+        </is>
+      </c>
+      <c r="M80" s="20" t="inlineStr">
+        <is>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="N80" s="14" t="inlineStr">
@@ -4100,24 +4052,24 @@
       </c>
     </row>
     <row r="81" ht="22" customHeight="1">
-      <c r="A81" s="34" t="inlineStr">
+      <c r="A81" s="30" t="inlineStr">
         <is>
           <t>DS_25 — Trang Quên mật khẩu   (5 lỗi: 5 đã xử lý, 0 đang mở)</t>
         </is>
       </c>
-      <c r="B81" s="35" t="n"/>
-      <c r="C81" s="35" t="n"/>
-      <c r="D81" s="35" t="n"/>
-      <c r="E81" s="35" t="n"/>
-      <c r="F81" s="35" t="n"/>
-      <c r="G81" s="35" t="n"/>
-      <c r="H81" s="35" t="n"/>
-      <c r="I81" s="35" t="n"/>
-      <c r="J81" s="35" t="n"/>
-      <c r="K81" s="35" t="n"/>
-      <c r="L81" s="35" t="n"/>
-      <c r="M81" s="35" t="n"/>
-      <c r="N81" s="35" t="n"/>
+      <c r="B81" s="31" t="n"/>
+      <c r="C81" s="31" t="n"/>
+      <c r="D81" s="31" t="n"/>
+      <c r="E81" s="31" t="n"/>
+      <c r="F81" s="31" t="n"/>
+      <c r="G81" s="31" t="n"/>
+      <c r="H81" s="31" t="n"/>
+      <c r="I81" s="31" t="n"/>
+      <c r="J81" s="31" t="n"/>
+      <c r="K81" s="31" t="n"/>
+      <c r="L81" s="31" t="n"/>
+      <c r="M81" s="31" t="n"/>
+      <c r="N81" s="31" t="n"/>
     </row>
     <row r="82" ht="30" customHeight="1">
       <c r="A82" s="13" t="inlineStr">
@@ -4797,7 +4749,7 @@
       </c>
       <c r="B99" s="10" t="inlineStr">
         <is>
-          <t>BUG_UI_107 (DS_22, Critical) đang mở: màu chìm trong template mail kích hoạt, chưa retest.</t>
+          <t>Toàn bộ lỗi trong phạm vi đã được Dev xử lý và QA retest đạt (Kết quả Retest = Pass). BUG_UI_107 trên DS_22 — lỗi cuối cùng còn mở — đã được đóng và retest Pass ngày 17/09/2026.</t>
         </is>
       </c>
       <c r="C99" s="11" t="n"/>
@@ -4806,13 +4758,13 @@
       <c r="F99" s="11" t="n"/>
       <c r="G99" s="10" t="inlineStr">
         <is>
-          <t>Chặn nghiệm thu DS_22</t>
+          <t>Không còn vướng mắc</t>
         </is>
       </c>
       <c r="H99" s="11" t="n"/>
-      <c r="I99" s="30" t="inlineStr"/>
-      <c r="J99" s="30" t="inlineStr"/>
-      <c r="K99" s="30" t="inlineStr"/>
+      <c r="I99" s="27" t="inlineStr"/>
+      <c r="J99" s="27" t="inlineStr"/>
+      <c r="K99" s="27" t="inlineStr"/>
       <c r="L99" s="9" t="n"/>
       <c r="M99" s="8" t="inlineStr"/>
       <c r="N99" s="9" t="n"/>
@@ -4823,7 +4775,7 @@
       </c>
       <c r="B100" s="15" t="inlineStr">
         <is>
-          <t>BUG_UI_107 được gắn YC_06 — tính năng này không nằm trong phạm vi DS_22 đã chốt (YC_04, YC_05, YC_07). Cần gắn lại đúng YC hoặc bổ sung YC_06 vào phạm vi.</t>
+          <t>BUG_UI_107 được gắn YC_06 (Xác minh email / Zalo) — tính năng này không nằm trong phạm vi DS_22 đã chốt (YC_04, YC_05, YC_07). Đề nghị gắn lại đúng YC hoặc bổ sung YC_06 vào phạm vi để hồ sơ thống nhất.</t>
         </is>
       </c>
       <c r="C100" s="16" t="n"/>
@@ -4832,13 +4784,13 @@
       <c r="F100" s="16" t="n"/>
       <c r="G100" s="15" t="inlineStr">
         <is>
-          <t>Ảnh hưởng cách tính phạm vi</t>
+          <t>Không đổi kết luận</t>
         </is>
       </c>
       <c r="H100" s="16" t="n"/>
-      <c r="I100" s="30" t="inlineStr"/>
-      <c r="J100" s="30" t="inlineStr"/>
-      <c r="K100" s="30" t="inlineStr"/>
+      <c r="I100" s="27" t="inlineStr"/>
+      <c r="J100" s="27" t="inlineStr"/>
+      <c r="K100" s="27" t="inlineStr"/>
       <c r="L100" s="9" t="n"/>
       <c r="M100" s="8" t="inlineStr"/>
       <c r="N100" s="9" t="n"/>
@@ -4849,7 +4801,7 @@
       </c>
       <c r="B101" s="10" t="inlineStr">
         <is>
-          <t>YC_04 còn 5 lỗi trên DS_23 (BUG_FUNC_020 đang sửa, BUG_REQ_002 Deferred). Theo phạm vi đã chốt, phần này thuộc đợt nghiệm thu sau.</t>
+          <t>YC_04 còn 5 lỗi trên DS_23 (BUG_FUNC_020 đang sửa, BUG_REQ_002 Deferred). Theo phạm vi đã chốt, phần YC_04 trên DS_23 thuộc đợt nghiệm thu sau.</t>
         </is>
       </c>
       <c r="C101" s="11" t="n"/>
@@ -4858,13 +4810,13 @@
       <c r="F101" s="11" t="n"/>
       <c r="G101" s="10" t="inlineStr">
         <is>
-          <t>Không chặn đợt này</t>
+          <t>Ngoài phạm vi đợt này</t>
         </is>
       </c>
       <c r="H101" s="11" t="n"/>
-      <c r="I101" s="30" t="inlineStr"/>
-      <c r="J101" s="30" t="inlineStr"/>
-      <c r="K101" s="30" t="inlineStr"/>
+      <c r="I101" s="27" t="inlineStr"/>
+      <c r="J101" s="27" t="inlineStr"/>
+      <c r="K101" s="27" t="inlineStr"/>
       <c r="L101" s="9" t="n"/>
       <c r="M101" s="8" t="inlineStr"/>
       <c r="N101" s="9" t="n"/>
@@ -4875,7 +4827,7 @@
       </c>
       <c r="B102" s="15" t="inlineStr">
         <is>
-          <t>3 lỗi chức năng không có ảnh bằng chứng (BUG_REG_001, BUG_FUNC_016, BUG_FUNC_019) — xác nhận bằng Kết quả Retest = Pass.</t>
+          <t>3 lỗi chức năng không có ảnh bằng chứng (BUG_REG_001, BUG_FUNC_016, BUG_FUNC_019) — hai bên thống nhất xác nhận bằng Kết quả Retest = Pass.</t>
         </is>
       </c>
       <c r="C102" s="16" t="n"/>
@@ -4884,13 +4836,13 @@
       <c r="F102" s="16" t="n"/>
       <c r="G102" s="15" t="inlineStr">
         <is>
-          <t>Không chặn — đã thống nhất</t>
+          <t>Đã thống nhất</t>
         </is>
       </c>
       <c r="H102" s="16" t="n"/>
-      <c r="I102" s="30" t="inlineStr"/>
-      <c r="J102" s="30" t="inlineStr"/>
-      <c r="K102" s="30" t="inlineStr"/>
+      <c r="I102" s="27" t="inlineStr"/>
+      <c r="J102" s="27" t="inlineStr"/>
+      <c r="K102" s="27" t="inlineStr"/>
       <c r="L102" s="9" t="n"/>
       <c r="M102" s="8" t="inlineStr"/>
       <c r="N102" s="9" t="n"/>
@@ -4901,7 +4853,7 @@
       </c>
       <c r="B103" s="10" t="inlineStr">
         <is>
-          <t>DS_22 chỉ có 1 Test Case và đang ở trạng thái Fail; DS_04, DS_21, DS_25 còn Test Case ở trạng thái Đang tiến hành.</t>
+          <t>DS_22 chỉ có 1 Test Case và đang ở trạng thái Fail; DS_04, DS_21, DS_25 còn Test Case ở trạng thái Đang tiến hành. Sheet 03_Test_Execution chưa có dữ liệu.</t>
         </is>
       </c>
       <c r="C103" s="11" t="n"/>
@@ -4910,13 +4862,13 @@
       <c r="F103" s="11" t="n"/>
       <c r="G103" s="10" t="inlineStr">
         <is>
-          <t>Cần hoàn tất trước khi mở rộng phạm vi</t>
+          <t>Cần hoàn tất trước đợt sau</t>
         </is>
       </c>
       <c r="H103" s="11" t="n"/>
-      <c r="I103" s="30" t="inlineStr"/>
-      <c r="J103" s="30" t="inlineStr"/>
-      <c r="K103" s="30" t="inlineStr"/>
+      <c r="I103" s="27" t="inlineStr"/>
+      <c r="J103" s="27" t="inlineStr"/>
+      <c r="K103" s="27" t="inlineStr"/>
       <c r="L103" s="9" t="n"/>
       <c r="M103" s="8" t="inlineStr"/>
       <c r="N103" s="9" t="n"/>
@@ -4940,9 +4892,9 @@
         </is>
       </c>
       <c r="H104" s="16" t="n"/>
-      <c r="I104" s="30" t="inlineStr"/>
-      <c r="J104" s="30" t="inlineStr"/>
-      <c r="K104" s="30" t="inlineStr"/>
+      <c r="I104" s="27" t="inlineStr"/>
+      <c r="J104" s="27" t="inlineStr"/>
+      <c r="K104" s="27" t="inlineStr"/>
       <c r="L104" s="9" t="n"/>
       <c r="M104" s="8" t="inlineStr"/>
       <c r="N104" s="9" t="n"/>
@@ -4953,7 +4905,7 @@
       </c>
       <c r="B105" s="10" t="inlineStr">
         <is>
-          <t>Công thức Tổng lỗi/Lỗi đã xử lý tại 02_UI_UX đếm cả dòng 'Không lỗi' (không có BUG_ID) nên bị đội số: DS_21 hiển thị 5 (thực tế 3), DS_22 hiển thị 4 (thực tế 2), DS_25 hiển thị 6 (thực tế 5). Toàn site có 29 dòng như vậy.</t>
+          <t>Công thức Tổng lỗi / Lỗi đã xử lý tại 02_UI_UX đếm cả dòng 'Không lỗi' (không có BUG_ID) nên bị đội số: DS_21 hiển thị 5 (thực tế 3), DS_22 hiển thị 4 (thực tế 2), DS_25 hiển thị 6 (thực tế 5). Toàn site có 29 dòng như vậy. Biên bản này dùng số thực tế đếm theo BUG_ID.</t>
         </is>
       </c>
       <c r="C105" s="11" t="n"/>
@@ -4966,9 +4918,9 @@
         </is>
       </c>
       <c r="H105" s="11" t="n"/>
-      <c r="I105" s="30" t="inlineStr"/>
-      <c r="J105" s="30" t="inlineStr"/>
-      <c r="K105" s="30" t="inlineStr"/>
+      <c r="I105" s="27" t="inlineStr"/>
+      <c r="J105" s="27" t="inlineStr"/>
+      <c r="K105" s="27" t="inlineStr"/>
       <c r="L105" s="9" t="n"/>
       <c r="M105" s="8" t="inlineStr"/>
       <c r="N105" s="9" t="n"/>
@@ -4995,40 +4947,40 @@
       <c r="N107" s="6" t="n"/>
     </row>
     <row r="108" ht="32" customHeight="1">
-      <c r="A108" s="37" t="inlineStr">
+      <c r="A108" s="32" t="inlineStr">
         <is>
           <t>Kết quả tự đánh giá theo tiêu chí mục III</t>
         </is>
       </c>
       <c r="B108" s="11" t="n"/>
       <c r="C108" s="11" t="n"/>
-      <c r="D108" s="38" t="inlineStr">
-        <is>
-          <t>4/5 màn hình ĐẠT nghiệm thu: DS_04, DS_05, DS_21, DS_25. CHƯA ĐẠT: DS_22 (Còn 1 lỗi đang mở; Còn 1 lỗi Critical/High chưa đóng)</t>
-        </is>
-      </c>
-      <c r="E108" s="23" t="n"/>
-      <c r="F108" s="23" t="n"/>
-      <c r="G108" s="23" t="n"/>
-      <c r="H108" s="23" t="n"/>
-      <c r="I108" s="23" t="n"/>
-      <c r="J108" s="23" t="n"/>
-      <c r="K108" s="23" t="n"/>
-      <c r="L108" s="23" t="n"/>
-      <c r="M108" s="23" t="n"/>
-      <c r="N108" s="23" t="n"/>
+      <c r="D108" s="33" t="inlineStr">
+        <is>
+          <t>5/5 màn hình ĐẠT nghiệm thu: DS_04, DS_05, DS_21, DS_22, DS_25. Không còn màn hình nào chưa đạt. Đề xuất kết luận: ĐẠT NGHIỆM THU GIAI ĐOẠN 1.</t>
+        </is>
+      </c>
+      <c r="E108" s="21" t="n"/>
+      <c r="F108" s="21" t="n"/>
+      <c r="G108" s="21" t="n"/>
+      <c r="H108" s="21" t="n"/>
+      <c r="I108" s="21" t="n"/>
+      <c r="J108" s="21" t="n"/>
+      <c r="K108" s="21" t="n"/>
+      <c r="L108" s="21" t="n"/>
+      <c r="M108" s="21" t="n"/>
+      <c r="N108" s="21" t="n"/>
     </row>
     <row r="109" ht="28" customHeight="1">
-      <c r="A109" s="37" t="inlineStr">
-        <is>
-          <t>Điều kiện để DS_22 được nghiệm thu</t>
+      <c r="A109" s="32" t="inlineStr">
+        <is>
+          <t>Ghi nhận</t>
         </is>
       </c>
       <c r="B109" s="11" t="n"/>
       <c r="C109" s="11" t="n"/>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>Dev đóng BUG_UI_107, QA retest đạt và cập nhật Kết quả Retest = Pass; sau đó DS_22 đủ 4 điều kiện và được ký cùng 4 màn hình còn lại.</t>
+          <t>Toàn bộ 5 màn hình và 12 tính năng trong phạm vi đã thỏa mãn 6 tiêu chí tại mục III. 19/19 lỗi đã được xử lý và retest đạt. Hồ sơ đủ điều kiện trình ký.</t>
         </is>
       </c>
       <c r="E109" s="11" t="n"/>
@@ -5043,35 +4995,35 @@
       <c r="N109" s="11" t="n"/>
     </row>
     <row r="110" ht="30" customHeight="1">
-      <c r="A110" s="39" t="inlineStr">
+      <c r="A110" s="34" t="inlineStr">
         <is>
           <t>KẾT LUẬN CHÍNH THỨC (người duyệt ghi)</t>
         </is>
       </c>
-      <c r="B110" s="40" t="n"/>
-      <c r="C110" s="40" t="n"/>
-      <c r="D110" s="41" t="inlineStr"/>
+      <c r="B110" s="35" t="n"/>
+      <c r="C110" s="35" t="n"/>
+      <c r="D110" s="36" t="inlineStr"/>
       <c r="E110" s="9" t="n"/>
       <c r="F110" s="9" t="n"/>
       <c r="G110" s="9" t="n"/>
-      <c r="H110" s="42" t="inlineStr">
+      <c r="H110" s="37" t="inlineStr">
         <is>
           <t>Ngày kết luận</t>
         </is>
       </c>
-      <c r="I110" s="30" t="inlineStr"/>
+      <c r="I110" s="27" t="inlineStr"/>
       <c r="J110" s="9" t="n"/>
-      <c r="K110" s="42" t="inlineStr">
+      <c r="K110" s="37" t="inlineStr">
         <is>
           <t>Hiệu lực từ</t>
         </is>
       </c>
-      <c r="L110" s="30" t="inlineStr"/>
+      <c r="L110" s="27" t="inlineStr"/>
       <c r="M110" s="9" t="n"/>
       <c r="N110" s="9" t="n"/>
     </row>
     <row r="111" ht="44" customHeight="1">
-      <c r="A111" s="37" t="inlineStr">
+      <c r="A111" s="32" t="inlineStr">
         <is>
           <t>Ý kiến / điều kiện kèm theo</t>
         </is>
@@ -5172,19 +5124,19 @@
       <c r="N115" s="12" t="inlineStr"/>
     </row>
     <row r="116" ht="52" customHeight="1">
-      <c r="A116" s="43" t="inlineStr">
+      <c r="A116" s="38" t="inlineStr">
         <is>
           <t>ĐẠI DIỆN BÊN A (Chủ đầu tư)</t>
         </is>
       </c>
       <c r="B116" s="11" t="n"/>
-      <c r="C116" s="30" t="inlineStr"/>
+      <c r="C116" s="27" t="inlineStr"/>
       <c r="D116" s="9" t="n"/>
-      <c r="E116" s="30" t="inlineStr"/>
+      <c r="E116" s="27" t="inlineStr"/>
       <c r="F116" s="8" t="inlineStr"/>
       <c r="G116" s="9" t="n"/>
       <c r="H116" s="9" t="n"/>
-      <c r="I116" s="30" t="inlineStr"/>
+      <c r="I116" s="27" t="inlineStr"/>
       <c r="J116" s="13" t="inlineStr"/>
       <c r="K116" s="11" t="n"/>
       <c r="L116" s="11" t="n"/>
@@ -5192,19 +5144,19 @@
       <c r="N116" s="11" t="n"/>
     </row>
     <row r="117" ht="52" customHeight="1">
-      <c r="A117" s="44" t="inlineStr">
+      <c r="A117" s="39" t="inlineStr">
         <is>
           <t>ĐẠI DIỆN BÊN B (Đơn vị thực hiện)</t>
         </is>
       </c>
       <c r="B117" s="16" t="n"/>
-      <c r="C117" s="30" t="inlineStr"/>
+      <c r="C117" s="27" t="inlineStr"/>
       <c r="D117" s="9" t="n"/>
-      <c r="E117" s="30" t="inlineStr"/>
+      <c r="E117" s="27" t="inlineStr"/>
       <c r="F117" s="8" t="inlineStr"/>
       <c r="G117" s="9" t="n"/>
       <c r="H117" s="9" t="n"/>
-      <c r="I117" s="30" t="inlineStr"/>
+      <c r="I117" s="27" t="inlineStr"/>
       <c r="J117" s="14" t="inlineStr"/>
       <c r="K117" s="16" t="n"/>
       <c r="L117" s="16" t="n"/>
@@ -5212,19 +5164,19 @@
       <c r="N117" s="16" t="n"/>
     </row>
     <row r="118" ht="52" customHeight="1">
-      <c r="A118" s="43" t="inlineStr">
+      <c r="A118" s="38" t="inlineStr">
         <is>
           <t>QUẢN LÝ DỰ ÁN</t>
         </is>
       </c>
       <c r="B118" s="11" t="n"/>
-      <c r="C118" s="30" t="inlineStr"/>
+      <c r="C118" s="27" t="inlineStr"/>
       <c r="D118" s="9" t="n"/>
-      <c r="E118" s="30" t="inlineStr"/>
+      <c r="E118" s="27" t="inlineStr"/>
       <c r="F118" s="8" t="inlineStr"/>
       <c r="G118" s="9" t="n"/>
       <c r="H118" s="9" t="n"/>
-      <c r="I118" s="30" t="inlineStr"/>
+      <c r="I118" s="27" t="inlineStr"/>
       <c r="J118" s="13" t="inlineStr"/>
       <c r="K118" s="11" t="n"/>
       <c r="L118" s="11" t="n"/>
@@ -5232,19 +5184,19 @@
       <c r="N118" s="11" t="n"/>
     </row>
     <row r="119" ht="52" customHeight="1">
-      <c r="A119" s="44" t="inlineStr">
+      <c r="A119" s="39" t="inlineStr">
         <is>
           <t>QA / TESTER</t>
         </is>
       </c>
       <c r="B119" s="16" t="n"/>
-      <c r="C119" s="30" t="inlineStr"/>
+      <c r="C119" s="27" t="inlineStr"/>
       <c r="D119" s="9" t="n"/>
-      <c r="E119" s="30" t="inlineStr"/>
+      <c r="E119" s="27" t="inlineStr"/>
       <c r="F119" s="8" t="inlineStr"/>
       <c r="G119" s="9" t="n"/>
       <c r="H119" s="9" t="n"/>
-      <c r="I119" s="30" t="inlineStr"/>
+      <c r="I119" s="27" t="inlineStr"/>
       <c r="J119" s="14" t="inlineStr"/>
       <c r="K119" s="16" t="n"/>
       <c r="L119" s="16" t="n"/>
@@ -5252,19 +5204,19 @@
       <c r="N119" s="16" t="n"/>
     </row>
     <row r="120" ht="52" customHeight="1">
-      <c r="A120" s="43" t="inlineStr">
+      <c r="A120" s="38" t="inlineStr">
         <is>
           <t>ĐẠI DIỆN DEV</t>
         </is>
       </c>
       <c r="B120" s="11" t="n"/>
-      <c r="C120" s="30" t="inlineStr"/>
+      <c r="C120" s="27" t="inlineStr"/>
       <c r="D120" s="9" t="n"/>
-      <c r="E120" s="30" t="inlineStr"/>
+      <c r="E120" s="27" t="inlineStr"/>
       <c r="F120" s="8" t="inlineStr"/>
       <c r="G120" s="9" t="n"/>
       <c r="H120" s="9" t="n"/>
-      <c r="I120" s="30" t="inlineStr"/>
+      <c r="I120" s="27" t="inlineStr"/>
       <c r="J120" s="13" t="inlineStr"/>
       <c r="K120" s="11" t="n"/>
       <c r="L120" s="11" t="n"/>
@@ -5326,14 +5278,14 @@
           <t>PL-01</t>
         </is>
       </c>
-      <c r="B124" s="45" t="inlineStr">
+      <c r="B124" s="40" t="inlineStr">
         <is>
           <t>Danh sách lỗi đầy đủ kèm link bằng chứng</t>
         </is>
       </c>
       <c r="C124" s="11" t="n"/>
       <c r="D124" s="11" t="n"/>
-      <c r="E124" s="45" t="inlineStr">
+      <c r="E124" s="40" t="inlineStr">
         <is>
           <t>File QA — sheet 05_Lỗi_Tester</t>
         </is>
@@ -5354,14 +5306,14 @@
           <t>PL-02</t>
         </is>
       </c>
-      <c r="B125" s="46" t="inlineStr">
+      <c r="B125" s="41" t="inlineStr">
         <is>
           <t>Tình trạng xử lý và retest của Dev</t>
         </is>
       </c>
       <c r="C125" s="16" t="n"/>
       <c r="D125" s="16" t="n"/>
-      <c r="E125" s="46" t="inlineStr">
+      <c r="E125" s="41" t="inlineStr">
         <is>
           <t>File QA — sheet 06_RTM_Dev_Test</t>
         </is>
@@ -5382,14 +5334,14 @@
           <t>PL-03</t>
         </is>
       </c>
-      <c r="B126" s="45" t="inlineStr">
+      <c r="B126" s="40" t="inlineStr">
         <is>
           <t>Trạng thái kiểm thử theo trang</t>
         </is>
       </c>
       <c r="C126" s="11" t="n"/>
       <c r="D126" s="11" t="n"/>
-      <c r="E126" s="45" t="inlineStr">
+      <c r="E126" s="40" t="inlineStr">
         <is>
           <t>File QA — sheet 02_UI_UX</t>
         </is>
@@ -5410,14 +5362,14 @@
           <t>PL-04</t>
         </is>
       </c>
-      <c r="B127" s="46" t="inlineStr">
+      <c r="B127" s="41" t="inlineStr">
         <is>
           <t>Trạng thái kiểm thử theo tính năng</t>
         </is>
       </c>
       <c r="C127" s="16" t="n"/>
       <c r="D127" s="16" t="n"/>
-      <c r="E127" s="46" t="inlineStr">
+      <c r="E127" s="41" t="inlineStr">
         <is>
           <t>File QA — sheet 03_Tính_năng</t>
         </is>
@@ -5438,14 +5390,14 @@
           <t>PL-05</t>
         </is>
       </c>
-      <c r="B128" s="45" t="inlineStr">
+      <c r="B128" s="40" t="inlineStr">
         <is>
           <t>Bộ Test Case liên quan</t>
         </is>
       </c>
       <c r="C128" s="11" t="n"/>
       <c r="D128" s="11" t="n"/>
-      <c r="E128" s="45" t="inlineStr">
+      <c r="E128" s="40" t="inlineStr">
         <is>
           <t>File QA — sheet 04_Test_Cases</t>
         </is>

</xml_diff>